<commit_message>
Add optional CPU scene analysis, OCR frame review and 25-case test sheet
</commit_message>
<xml_diff>
--- a/docs/SceneForge_BangThuThat_DoiChieu.xlsx
+++ b/docs/SceneForge_BangThuThat_DoiChieu.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="9" min="1" max="1"/>
@@ -1784,6 +1784,162 @@
       <c r="J29" s="18" t="inlineStr">
         <is>
           <t>Có Notification API và âm báo; chưa thử thông báo hệ điều hành khi thu nhỏ trên Windows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>🟠 Cần số thật</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Phân tích · máy</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>faster-whisper chép tiếng Trung có chuẩn không</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>0đ</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>Chạy faster-whisper trên 3 video mẫu tiếng Trung, so lời và mốc giây với video.</t>
+        </is>
+      </c>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>Lời đúng, mốc giây lệch không quá rõ khi xem.</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>Để Gemini chép lời như cũ, faster-whisper chỉ dùng để lấy mốc giây.</t>
+        </is>
+      </c>
+      <c r="I30" s="18" t="inlineStr">
+        <is>
+          <t>Chưa thử</t>
+        </is>
+      </c>
+      <c r="J30" s="18" t="inlineStr">
+        <is>
+          <t>Chưa thử tiêu chí video thật. Xem aggregate-2-implementation.md: có adapter / fixture cục bộ, không chứng nhận D5–D7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>🔴 Làm trước</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Phân tích · máy</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>PySceneDetect cắt có khớp video TikTok cắt nhanh không</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>0đ</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Chạy trên 5 video mẫu, so số cảnh và mốc cắt với mắt nhìn.</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Không sót, không thừa chỗ cắt rõ ràng.</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Chỉnh độ nhạy, hoặc để sau thêm TransNetV2.</t>
+        </is>
+      </c>
+      <c r="I31" s="18" t="inlineStr">
+        <is>
+          <t>Chưa thử</t>
+        </is>
+      </c>
+      <c r="J31" s="18" t="inlineStr">
+        <is>
+          <t>Chưa thử tiêu chí video thật. Xem aggregate-2-implementation.md: có adapter / fixture cục bộ, không chứng nhận D5–D7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>🟡 Nhỏ</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>Phân tích · máy</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Che logo trên khung gốc bằng OpenCV có sạch không</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>0đ</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>Lấy 3 khung có logo đối thủ, cho RapidOCR tìm và OpenCV tô lấp.</t>
+        </is>
+      </c>
+      <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>Nhìn không thấy vệt rõ.</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>Gửi Flow sửa ảnh (0 credit theo bảng giá hiện tại).</t>
+        </is>
+      </c>
+      <c r="I32" s="18" t="inlineStr">
+        <is>
+          <t>Chưa thử</t>
+        </is>
+      </c>
+      <c r="J32" s="18" t="inlineStr">
+        <is>
+          <t>Chưa thử tiêu chí video thật. Xem aggregate-2-implementation.md: có adapter / fixture cục bộ, không chứng nhận D5–D7.</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="10" min="1" max="1"/>
@@ -1976,6 +2132,40 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CPU cảnh/OCR/ảnh</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Đạt fixture tổng hợp</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cắt 1s, OCR BRAND, chọn vùng/xem/lưu bản ảnh mới chưa duyệt; xem trước/reload/giữ clip/hoàn tác. Không dùng thay D5–D7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Whisper model thật</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Chưa thử</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Adapter CPU int8 + mốc từ đã nối; tải model bị proxy 403, không giả kết quả suy luận.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>